<commit_message>
backend: admin dashboard part B (results, exports, reset, audit log)
- Standings service: per-category ranking (shared ranks for ties,
  zero-vote exhibitors included, votes for removed exhibitors kept);
  same shape as the planned GET /results
- live results widget on the dashboard, refreshed every 5 seconds
- results CSV export (F13) and visitor CSV export (F14) with a
  personal-data warning; cells protected against formula injection
- reset results: only while voting is closed, slug confirmation,
  deletes only this event's votes
- read-only audit log page; admin sign-ins and failed sign-ins audited
- ERD doc and exports updated for the Filament MFA columns

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/export/erd.xlsx
+++ b/docs/export/erd.xlsx
@@ -655,7 +655,7 @@
       </c>
       <c r="B15" s="4" t="inlineStr">
         <is>
-          <t>One pool of admins (users); every admin can manage every event. MFA (TOTP) enrolled via two_factor_*.</t>
+          <t>One pool of admins (users); every admin can manage every event. MFA (TOTP, required) stored in app_authentication_secret + recovery codes.</t>
         </is>
       </c>
     </row>
@@ -2728,7 +2728,7 @@
       </c>
       <c r="B65" s="6" t="inlineStr">
         <is>
-          <t>two_factor_secret</t>
+          <t>app_authentication_secret</t>
         </is>
       </c>
       <c r="C65" s="6" t="inlineStr">
@@ -2744,7 +2744,7 @@
       </c>
       <c r="F65" s="4" t="inlineStr">
         <is>
-          <t>TOTP secret, encrypted</t>
+          <t>TOTP secret for the authenticator app, encrypted (Filament MFA)</t>
         </is>
       </c>
     </row>
@@ -2756,12 +2756,12 @@
       </c>
       <c r="B66" s="6" t="inlineStr">
         <is>
-          <t>two_factor_confirmed_at</t>
+          <t>app_authentication_recovery_codes</t>
         </is>
       </c>
       <c r="C66" s="6" t="inlineStr">
         <is>
-          <t>timestamptz</t>
+          <t>text</t>
         </is>
       </c>
       <c r="D66" s="7" t="inlineStr"/>
@@ -2772,7 +2772,7 @@
       </c>
       <c r="F66" s="4" t="inlineStr">
         <is>
-          <t>MFA enrolled</t>
+          <t>One-time recovery codes, encrypted</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
backend: max 3 categories per event, one category per exhibitor
- exhibitors.category_id replaces the category_exhibitor pivot; the
  migration keeps each exhibitor's first category and refuses to run
  if that would separate existing votes
- database: the category must belong to the exhibitor's event, and
  votes reference exhibitors(event_id, category_id, id) ON UPDATE
  RESTRICT, so an exhibitor with votes cannot change category
- Category model caps an event at voting.max_categories_per_event (3)
- admin: "New category" disabled at the limit; single category select,
  locked once the exhibitor has votes; category filter; categories
  with exhibitors cannot be deleted
- standings, seeder, factories and tests updated
- docs: ERD and API contract record the decision (spec F9 allowed
  one or more); exports regenerated

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/export/erd.xlsx
+++ b/docs/export/erd.xlsx
@@ -14,10 +14,10 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Constraints &amp; Indexes" sheetId="5" state="visible" r:id="rId5"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Tables'!$A$1:$C$11</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Columns'!$A$1:$F$73</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Relationships'!$A$1:$F$14</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Constraints &amp; Indexes'!$A$1:$D$19</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Tables'!$A$1:$C$10</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Columns'!$A$1:$F$71</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Relationships'!$A$1:$F$13</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Constraints &amp; Indexes'!$A$1:$D$18</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -494,7 +494,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B17"/>
+  <dimension ref="A1:B18"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="28" customWidth="1" min="1" max="1"/>
@@ -535,7 +535,7 @@
       </c>
       <c r="B5" s="4" t="inlineStr">
         <is>
-          <t>Implemented in backend/database/migrations and running on Supabase (revision 3). Source of truth: docs/02-erd.md</t>
+          <t>Implemented in backend/database/migrations and running on Supabase (revision 4). Source of truth: docs/02-erd.md</t>
         </is>
       </c>
     </row>
@@ -602,82 +602,94 @@
     <row r="11">
       <c r="A11" s="3" t="inlineStr">
         <is>
-          <t>Same-event integrity</t>
+          <t>Categories</t>
         </is>
       </c>
       <c r="B11" s="4" t="inlineStr">
         <is>
-          <t>Composite foreign keys (event_id, ...) guarantee categories, exhibitors, registrations and votes of an event can never point at another event's rows.</t>
+          <t>At most 3 categories per event; each exhibitor competes in exactly one category (decision; spec F9 allowed one or more).</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="3" t="inlineStr">
         <is>
-          <t>Voting open rule</t>
+          <t>Same-event integrity</t>
         </is>
       </c>
       <c r="B12" s="4" t="inlineStr">
         <is>
-          <t>voting_enabled = true AND (opens_at is null OR now &gt;= opens_at) AND (closes_at is null OR now &lt; closes_at)</t>
+          <t>Composite foreign keys (event_id, ...) guarantee categories, exhibitors, registrations and votes of an event can never point at another event's rows.</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="3" t="inlineStr">
         <is>
-          <t>One vote per category</t>
+          <t>Voting open rule</t>
         </is>
       </c>
       <c r="B13" s="4" t="inlineStr">
         <is>
-          <t>UNIQUE (visitor_id, category_id) on votes - enforced by the database (F2, F12). Votes are immutable.</t>
+          <t>voting_enabled = true AND (opens_at is null OR now &gt;= opens_at) AND (closes_at is null OR now &lt; closes_at)</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="3" t="inlineStr">
         <is>
-          <t>Privacy (F14)</t>
+          <t>One vote per category</t>
         </is>
       </c>
       <c r="B14" s="4" t="inlineStr">
         <is>
-          <t>Phone stored encrypted (phone_encrypted) + HMAC-SHA256 blind index (phone_hash) for uniqueness/lookup. RLS enabled with NO policies on every table so the public Supabase API cannot read data; Laravel is the only access path. anon/authenticated roles also have all table privileges revoked. OTP codes and tokens stored hashed.</t>
+          <t>UNIQUE (visitor_id, category_id) on votes - enforced by the database (F2, F12). Votes are immutable.</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="3" t="inlineStr">
         <is>
-          <t>Admins</t>
+          <t>Privacy (F14)</t>
         </is>
       </c>
       <c r="B15" s="4" t="inlineStr">
         <is>
-          <t>One pool of admins (users); every admin can manage every event. MFA (TOTP, required) stored in app_authentication_secret + recovery codes.</t>
+          <t>Phone stored encrypted (phone_encrypted) + HMAC-SHA256 blind index (phone_hash) for uniqueness/lookup. RLS enabled with NO policies on every table so the public Supabase API cannot read data; Laravel is the only access path. anon/authenticated roles also have all table privileges revoked. OTP codes and tokens stored hashed.</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="3" t="inlineStr">
         <is>
-          <t>Framework tables (not listed)</t>
+          <t>Admins</t>
         </is>
       </c>
       <c r="B16" s="4" t="inlineStr">
         <is>
-          <t>personal_access_tokens (Sanctum; visitor + display tokens, bound to one event via abilities), sessions, cache, cache_locks, jobs, failed_jobs - database-backed so the app stays stateless.</t>
+          <t>One pool of admins (users); every admin can manage every event. MFA (TOTP, required) stored in app_authentication_secret + recovery codes.</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="3" t="inlineStr">
         <is>
+          <t>Framework tables (not listed)</t>
+        </is>
+      </c>
+      <c r="B17" s="4" t="inlineStr">
+        <is>
+          <t>personal_access_tokens (Sanctum; visitor + display tokens, bound to one event via abilities), sessions, cache, cache_locks, jobs, failed_jobs - database-backed so the app stays stateless.</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="3" t="inlineStr">
+        <is>
           <t>Not drawn in the picture</t>
         </is>
       </c>
-      <c r="B17" s="4" t="inlineStr">
+      <c r="B18" s="4" t="inlineStr">
         <is>
           <t>votes.event_id -&gt; events.id and audit_logs.event_id -&gt; events.id exist (see Relationships tab).</t>
         </is>
@@ -694,7 +706,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C11"/>
+  <dimension ref="A1:C10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="24" customWidth="1" min="1" max="1"/>
@@ -773,41 +785,41 @@
     <row r="5">
       <c r="A5" s="6" t="inlineStr">
         <is>
-          <t>category_exhibitor</t>
+          <t>visitors</t>
         </is>
       </c>
       <c r="B5" s="4" t="inlineStr">
         <is>
-          <t>Per event</t>
+          <t>Global</t>
         </is>
       </c>
       <c r="C5" s="4" t="inlineStr">
         <is>
-          <t>Many-to-many: exhibitor entered in one or more categories of the same event.</t>
+          <t>One row per phone number = the visitor's UID (encrypted + blind index). Identity only - no verification state.</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="6" t="inlineStr">
         <is>
-          <t>visitors</t>
+          <t>event_registrations</t>
         </is>
       </c>
       <c r="B6" s="4" t="inlineStr">
         <is>
-          <t>Global</t>
+          <t>Per event</t>
         </is>
       </c>
       <c r="C6" s="4" t="inlineStr">
         <is>
-          <t>One row per phone number = the visitor's UID (encrypted + blind index). Identity only - no verification state.</t>
+          <t>A visitor's participation in ONE event; holds phone_verified_at, i.e. the per-event OTP confirmation.</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="6" t="inlineStr">
         <is>
-          <t>event_registrations</t>
+          <t>otp_codes</t>
         </is>
       </c>
       <c r="B7" s="4" t="inlineStr">
@@ -817,14 +829,14 @@
       </c>
       <c r="C7" s="4" t="inlineStr">
         <is>
-          <t>A visitor's participation in ONE event; holds phone_verified_at, i.e. the per-event OTP confirmation.</t>
+          <t>Hashed one-time codes, belonging to an event registration.</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="6" t="inlineStr">
         <is>
-          <t>otp_codes</t>
+          <t>votes</t>
         </is>
       </c>
       <c r="B8" s="4" t="inlineStr">
@@ -834,63 +846,46 @@
       </c>
       <c r="C8" s="4" t="inlineStr">
         <is>
-          <t>Hashed one-time codes, belonging to an event registration.</t>
+          <t>One row per cast vote; immutable; unique per visitor + category.</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="6" t="inlineStr">
         <is>
-          <t>votes</t>
+          <t>users</t>
         </is>
       </c>
       <c r="B9" s="4" t="inlineStr">
         <is>
-          <t>Per event</t>
+          <t>Global</t>
         </is>
       </c>
       <c r="C9" s="4" t="inlineStr">
         <is>
-          <t>One row per cast vote; immutable; unique per visitor + category.</t>
+          <t>Admins (Makerspace staff). Not visitors.</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="6" t="inlineStr">
         <is>
-          <t>users</t>
+          <t>audit_logs</t>
         </is>
       </c>
       <c r="B10" s="4" t="inlineStr">
         <is>
-          <t>Global</t>
+          <t>Global / per event</t>
         </is>
       </c>
       <c r="C10" s="4" t="inlineStr">
         <is>
-          <t>Admins (Makerspace staff). Not visitors.</t>
-        </is>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" s="6" t="inlineStr">
-        <is>
-          <t>audit_logs</t>
-        </is>
-      </c>
-      <c r="B11" s="4" t="inlineStr">
-        <is>
-          <t>Global / per event</t>
-        </is>
-      </c>
-      <c r="C11" s="4" t="inlineStr">
-        <is>
           <t>Append-only log of sensitive admin actions (reset, exports, settings).</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:C11"/>
+  <autoFilter ref="A1:C10"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -901,7 +896,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F73"/>
+  <dimension ref="A1:F71"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="24" customWidth="1" min="1" max="1"/>
@@ -1648,21 +1643,29 @@
       </c>
       <c r="B27" s="6" t="inlineStr">
         <is>
-          <t>name</t>
+          <t>category_id</t>
         </is>
       </c>
       <c r="C27" s="6" t="inlineStr">
         <is>
-          <t>varchar</t>
-        </is>
-      </c>
-      <c r="D27" s="7" t="inlineStr"/>
+          <t>bigint</t>
+        </is>
+      </c>
+      <c r="D27" s="7" t="inlineStr">
+        <is>
+          <t>FK</t>
+        </is>
+      </c>
       <c r="E27" s="7" t="inlineStr">
         <is>
           <t>no</t>
         </is>
       </c>
-      <c r="F27" s="4" t="inlineStr"/>
+      <c r="F27" s="4" t="inlineStr">
+        <is>
+          <t>The one category it competes in: (event_id, category_id) -&gt; categories(event_id, id)</t>
+        </is>
+      </c>
     </row>
     <row r="28">
       <c r="A28" s="6" t="inlineStr">
@@ -1672,12 +1675,12 @@
       </c>
       <c r="B28" s="6" t="inlineStr">
         <is>
-          <t>short_description</t>
+          <t>name</t>
         </is>
       </c>
       <c r="C28" s="6" t="inlineStr">
         <is>
-          <t>text</t>
+          <t>varchar</t>
         </is>
       </c>
       <c r="D28" s="7" t="inlineStr"/>
@@ -1686,11 +1689,7 @@
           <t>no</t>
         </is>
       </c>
-      <c r="F28" s="4" t="inlineStr">
-        <is>
-          <t>Shown on the voting card</t>
-        </is>
-      </c>
+      <c r="F28" s="4" t="inlineStr"/>
     </row>
     <row r="29">
       <c r="A29" s="6" t="inlineStr">
@@ -1700,23 +1699,23 @@
       </c>
       <c r="B29" s="6" t="inlineStr">
         <is>
-          <t>photo_path</t>
+          <t>short_description</t>
         </is>
       </c>
       <c r="C29" s="6" t="inlineStr">
         <is>
-          <t>varchar</t>
+          <t>text</t>
         </is>
       </c>
       <c r="D29" s="7" t="inlineStr"/>
       <c r="E29" s="7" t="inlineStr">
         <is>
-          <t>yes</t>
+          <t>no</t>
         </is>
       </c>
       <c r="F29" s="4" t="inlineStr">
         <is>
-          <t>Object key in Supabase Storage (S3-compatible); API builds the public URL</t>
+          <t>Shown on the voting card</t>
         </is>
       </c>
     </row>
@@ -1728,21 +1727,25 @@
       </c>
       <c r="B30" s="6" t="inlineStr">
         <is>
-          <t>is_active</t>
+          <t>photo_path</t>
         </is>
       </c>
       <c r="C30" s="6" t="inlineStr">
         <is>
-          <t>bool</t>
+          <t>varchar</t>
         </is>
       </c>
       <c r="D30" s="7" t="inlineStr"/>
       <c r="E30" s="7" t="inlineStr">
         <is>
-          <t>no</t>
-        </is>
-      </c>
-      <c r="F30" s="4" t="inlineStr"/>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="F30" s="4" t="inlineStr">
+        <is>
+          <t>Object key in Supabase Storage (S3-compatible); API builds the public URL</t>
+        </is>
+      </c>
     </row>
     <row r="31">
       <c r="A31" s="6" t="inlineStr">
@@ -1752,67 +1755,59 @@
       </c>
       <c r="B31" s="6" t="inlineStr">
         <is>
-          <t>deleted_at</t>
+          <t>is_active</t>
         </is>
       </c>
       <c r="C31" s="6" t="inlineStr">
         <is>
-          <t>timestamptz</t>
+          <t>bool</t>
         </is>
       </c>
       <c r="D31" s="7" t="inlineStr"/>
       <c r="E31" s="7" t="inlineStr">
         <is>
-          <t>yes</t>
-        </is>
-      </c>
-      <c r="F31" s="4" t="inlineStr">
-        <is>
-          <t>Soft delete; hard delete blocked once votes exist</t>
-        </is>
-      </c>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="F31" s="4" t="inlineStr"/>
     </row>
     <row r="32">
       <c r="A32" s="6" t="inlineStr">
         <is>
-          <t>category_exhibitor</t>
+          <t>exhibitors</t>
         </is>
       </c>
       <c r="B32" s="6" t="inlineStr">
         <is>
-          <t>event_id</t>
+          <t>deleted_at</t>
         </is>
       </c>
       <c r="C32" s="6" t="inlineStr">
         <is>
-          <t>bigint</t>
-        </is>
-      </c>
-      <c r="D32" s="7" t="inlineStr">
-        <is>
-          <t>FK</t>
-        </is>
-      </c>
+          <t>timestamptz</t>
+        </is>
+      </c>
+      <c r="D32" s="7" t="inlineStr"/>
       <c r="E32" s="7" t="inlineStr">
         <is>
-          <t>no</t>
+          <t>yes</t>
         </is>
       </c>
       <c r="F32" s="4" t="inlineStr">
         <is>
-          <t>Part of both composite FKs</t>
+          <t>Soft delete; hard delete blocked once votes exist</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" s="6" t="inlineStr">
         <is>
-          <t>category_exhibitor</t>
+          <t>visitors</t>
         </is>
       </c>
       <c r="B33" s="6" t="inlineStr">
         <is>
-          <t>category_id</t>
+          <t>id</t>
         </is>
       </c>
       <c r="C33" s="6" t="inlineStr">
@@ -1822,7 +1817,7 @@
       </c>
       <c r="D33" s="7" t="inlineStr">
         <is>
-          <t>PK, FK</t>
+          <t>PK</t>
         </is>
       </c>
       <c r="E33" s="7" t="inlineStr">
@@ -1830,33 +1825,25 @@
           <t>no</t>
         </is>
       </c>
-      <c r="F33" s="4" t="inlineStr">
-        <is>
-          <t>(event_id, category_id) -&gt; categories(event_id, id)</t>
-        </is>
-      </c>
+      <c r="F33" s="4" t="inlineStr"/>
     </row>
     <row r="34">
       <c r="A34" s="6" t="inlineStr">
         <is>
-          <t>category_exhibitor</t>
+          <t>visitors</t>
         </is>
       </c>
       <c r="B34" s="6" t="inlineStr">
         <is>
-          <t>exhibitor_id</t>
+          <t>full_name</t>
         </is>
       </c>
       <c r="C34" s="6" t="inlineStr">
         <is>
-          <t>bigint</t>
-        </is>
-      </c>
-      <c r="D34" s="7" t="inlineStr">
-        <is>
-          <t>PK, FK</t>
-        </is>
-      </c>
+          <t>varchar</t>
+        </is>
+      </c>
+      <c r="D34" s="7" t="inlineStr"/>
       <c r="E34" s="7" t="inlineStr">
         <is>
           <t>no</t>
@@ -1864,7 +1851,7 @@
       </c>
       <c r="F34" s="4" t="inlineStr">
         <is>
-          <t>(event_id, exhibitor_id) -&gt; exhibitors(event_id, id)</t>
+          <t>Latest full name from a VERIFIED registration (outreach list)</t>
         </is>
       </c>
     </row>
@@ -1876,25 +1863,25 @@
       </c>
       <c r="B35" s="6" t="inlineStr">
         <is>
-          <t>id</t>
+          <t>phone_encrypted</t>
         </is>
       </c>
       <c r="C35" s="6" t="inlineStr">
         <is>
-          <t>bigint</t>
-        </is>
-      </c>
-      <c r="D35" s="7" t="inlineStr">
-        <is>
-          <t>PK</t>
-        </is>
-      </c>
+          <t>text</t>
+        </is>
+      </c>
+      <c r="D35" s="7" t="inlineStr"/>
       <c r="E35" s="7" t="inlineStr">
         <is>
           <t>no</t>
         </is>
       </c>
-      <c r="F35" s="4" t="inlineStr"/>
+      <c r="F35" s="4" t="inlineStr">
+        <is>
+          <t>E.164 number, Laravel encrypted cast (app key). Admin context only</t>
+        </is>
+      </c>
     </row>
     <row r="36">
       <c r="A36" s="6" t="inlineStr">
@@ -1904,15 +1891,19 @@
       </c>
       <c r="B36" s="6" t="inlineStr">
         <is>
-          <t>full_name</t>
+          <t>phone_hash</t>
         </is>
       </c>
       <c r="C36" s="6" t="inlineStr">
         <is>
-          <t>varchar</t>
-        </is>
-      </c>
-      <c r="D36" s="7" t="inlineStr"/>
+          <t>char(64)</t>
+        </is>
+      </c>
+      <c r="D36" s="7" t="inlineStr">
+        <is>
+          <t>UNIQUE</t>
+        </is>
+      </c>
       <c r="E36" s="7" t="inlineStr">
         <is>
           <t>no</t>
@@ -1920,7 +1911,7 @@
       </c>
       <c r="F36" s="4" t="inlineStr">
         <is>
-          <t>Latest full name from a VERIFIED registration (outreach list)</t>
+          <t>HMAC-SHA256 of the E.164 number with a dedicated secret - blind index</t>
         </is>
       </c>
     </row>
@@ -1932,45 +1923,41 @@
       </c>
       <c r="B37" s="6" t="inlineStr">
         <is>
-          <t>phone_encrypted</t>
+          <t>created_at / updated_at</t>
         </is>
       </c>
       <c r="C37" s="6" t="inlineStr">
         <is>
-          <t>text</t>
+          <t>timestamptz</t>
         </is>
       </c>
       <c r="D37" s="7" t="inlineStr"/>
       <c r="E37" s="7" t="inlineStr">
         <is>
-          <t>no</t>
-        </is>
-      </c>
-      <c r="F37" s="4" t="inlineStr">
-        <is>
-          <t>E.164 number, Laravel encrypted cast (app key). Admin context only</t>
-        </is>
-      </c>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="F37" s="4" t="inlineStr"/>
     </row>
     <row r="38">
       <c r="A38" s="6" t="inlineStr">
         <is>
-          <t>visitors</t>
+          <t>event_registrations</t>
         </is>
       </c>
       <c r="B38" s="6" t="inlineStr">
         <is>
-          <t>phone_hash</t>
+          <t>id</t>
         </is>
       </c>
       <c r="C38" s="6" t="inlineStr">
         <is>
-          <t>char(64)</t>
+          <t>bigint</t>
         </is>
       </c>
       <c r="D38" s="7" t="inlineStr">
         <is>
-          <t>UNIQUE</t>
+          <t>PK</t>
         </is>
       </c>
       <c r="E38" s="7" t="inlineStr">
@@ -1978,35 +1965,39 @@
           <t>no</t>
         </is>
       </c>
-      <c r="F38" s="4" t="inlineStr">
-        <is>
-          <t>HMAC-SHA256 of the E.164 number with a dedicated secret - blind index</t>
-        </is>
-      </c>
+      <c r="F38" s="4" t="inlineStr"/>
     </row>
     <row r="39">
       <c r="A39" s="6" t="inlineStr">
         <is>
-          <t>visitors</t>
+          <t>event_registrations</t>
         </is>
       </c>
       <c r="B39" s="6" t="inlineStr">
         <is>
-          <t>created_at / updated_at</t>
+          <t>event_id</t>
         </is>
       </c>
       <c r="C39" s="6" t="inlineStr">
         <is>
-          <t>timestamptz</t>
-        </is>
-      </c>
-      <c r="D39" s="7" t="inlineStr"/>
+          <t>bigint</t>
+        </is>
+      </c>
+      <c r="D39" s="7" t="inlineStr">
+        <is>
+          <t>FK</t>
+        </is>
+      </c>
       <c r="E39" s="7" t="inlineStr">
         <is>
-          <t>yes</t>
-        </is>
-      </c>
-      <c r="F39" s="4" t="inlineStr"/>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="F39" s="4" t="inlineStr">
+        <is>
+          <t>-&gt; events.id</t>
+        </is>
+      </c>
     </row>
     <row r="40">
       <c r="A40" s="6" t="inlineStr">
@@ -2016,7 +2007,7 @@
       </c>
       <c r="B40" s="6" t="inlineStr">
         <is>
-          <t>id</t>
+          <t>visitor_id</t>
         </is>
       </c>
       <c r="C40" s="6" t="inlineStr">
@@ -2026,7 +2017,7 @@
       </c>
       <c r="D40" s="7" t="inlineStr">
         <is>
-          <t>PK</t>
+          <t>FK</t>
         </is>
       </c>
       <c r="E40" s="7" t="inlineStr">
@@ -2034,7 +2025,11 @@
           <t>no</t>
         </is>
       </c>
-      <c r="F40" s="4" t="inlineStr"/>
+      <c r="F40" s="4" t="inlineStr">
+        <is>
+          <t>-&gt; visitors.id</t>
+        </is>
+      </c>
     </row>
     <row r="41">
       <c r="A41" s="6" t="inlineStr">
@@ -2044,19 +2039,15 @@
       </c>
       <c r="B41" s="6" t="inlineStr">
         <is>
-          <t>event_id</t>
+          <t>full_name</t>
         </is>
       </c>
       <c r="C41" s="6" t="inlineStr">
         <is>
-          <t>bigint</t>
-        </is>
-      </c>
-      <c r="D41" s="7" t="inlineStr">
-        <is>
-          <t>FK</t>
-        </is>
-      </c>
+          <t>varchar</t>
+        </is>
+      </c>
+      <c r="D41" s="7" t="inlineStr"/>
       <c r="E41" s="7" t="inlineStr">
         <is>
           <t>no</t>
@@ -2064,7 +2055,7 @@
       </c>
       <c r="F41" s="4" t="inlineStr">
         <is>
-          <t>-&gt; events.id</t>
+          <t>Full name entered for this event; copied to visitors.full_name only after verification</t>
         </is>
       </c>
     </row>
@@ -2076,27 +2067,23 @@
       </c>
       <c r="B42" s="6" t="inlineStr">
         <is>
-          <t>visitor_id</t>
+          <t>phone_verified_at</t>
         </is>
       </c>
       <c r="C42" s="6" t="inlineStr">
         <is>
-          <t>bigint</t>
-        </is>
-      </c>
-      <c r="D42" s="7" t="inlineStr">
-        <is>
-          <t>FK</t>
-        </is>
-      </c>
+          <t>timestamptz</t>
+        </is>
+      </c>
+      <c r="D42" s="7" t="inlineStr"/>
       <c r="E42" s="7" t="inlineStr">
         <is>
-          <t>no</t>
+          <t>yes</t>
         </is>
       </c>
       <c r="F42" s="4" t="inlineStr">
         <is>
-          <t>-&gt; visitors.id</t>
+          <t>Set when THIS event's OTP is verified (F6)</t>
         </is>
       </c>
     </row>
@@ -2108,23 +2095,23 @@
       </c>
       <c r="B43" s="6" t="inlineStr">
         <is>
-          <t>full_name</t>
+          <t>registered_ip</t>
         </is>
       </c>
       <c r="C43" s="6" t="inlineStr">
         <is>
-          <t>varchar</t>
+          <t>inet</t>
         </is>
       </c>
       <c r="D43" s="7" t="inlineStr"/>
       <c r="E43" s="7" t="inlineStr">
         <is>
-          <t>no</t>
+          <t>yes</t>
         </is>
       </c>
       <c r="F43" s="4" t="inlineStr">
         <is>
-          <t>Full name entered for this event; copied to visitors.full_name only after verification</t>
+          <t>Audit</t>
         </is>
       </c>
     </row>
@@ -2136,7 +2123,7 @@
       </c>
       <c r="B44" s="6" t="inlineStr">
         <is>
-          <t>phone_verified_at</t>
+          <t>created_at / updated_at</t>
         </is>
       </c>
       <c r="C44" s="6" t="inlineStr">
@@ -2150,63 +2137,67 @@
           <t>yes</t>
         </is>
       </c>
-      <c r="F44" s="4" t="inlineStr">
-        <is>
-          <t>Set when THIS event's OTP is verified (F6)</t>
-        </is>
-      </c>
+      <c r="F44" s="4" t="inlineStr"/>
     </row>
     <row r="45">
       <c r="A45" s="6" t="inlineStr">
         <is>
-          <t>event_registrations</t>
+          <t>otp_codes</t>
         </is>
       </c>
       <c r="B45" s="6" t="inlineStr">
         <is>
-          <t>registered_ip</t>
+          <t>id</t>
         </is>
       </c>
       <c r="C45" s="6" t="inlineStr">
         <is>
-          <t>inet</t>
-        </is>
-      </c>
-      <c r="D45" s="7" t="inlineStr"/>
+          <t>bigint</t>
+        </is>
+      </c>
+      <c r="D45" s="7" t="inlineStr">
+        <is>
+          <t>PK</t>
+        </is>
+      </c>
       <c r="E45" s="7" t="inlineStr">
         <is>
-          <t>yes</t>
-        </is>
-      </c>
-      <c r="F45" s="4" t="inlineStr">
-        <is>
-          <t>Audit</t>
-        </is>
-      </c>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="F45" s="4" t="inlineStr"/>
     </row>
     <row r="46">
       <c r="A46" s="6" t="inlineStr">
         <is>
-          <t>event_registrations</t>
+          <t>otp_codes</t>
         </is>
       </c>
       <c r="B46" s="6" t="inlineStr">
         <is>
-          <t>created_at / updated_at</t>
+          <t>event_registration_id</t>
         </is>
       </c>
       <c r="C46" s="6" t="inlineStr">
         <is>
-          <t>timestamptz</t>
-        </is>
-      </c>
-      <c r="D46" s="7" t="inlineStr"/>
+          <t>bigint</t>
+        </is>
+      </c>
+      <c r="D46" s="7" t="inlineStr">
+        <is>
+          <t>FK</t>
+        </is>
+      </c>
       <c r="E46" s="7" t="inlineStr">
         <is>
-          <t>yes</t>
-        </is>
-      </c>
-      <c r="F46" s="4" t="inlineStr"/>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="F46" s="4" t="inlineStr">
+        <is>
+          <t>-&gt; event_registrations.id ON DELETE CASCADE</t>
+        </is>
+      </c>
     </row>
     <row r="47">
       <c r="A47" s="6" t="inlineStr">
@@ -2216,25 +2207,25 @@
       </c>
       <c r="B47" s="6" t="inlineStr">
         <is>
-          <t>id</t>
+          <t>code_hash</t>
         </is>
       </c>
       <c r="C47" s="6" t="inlineStr">
         <is>
-          <t>bigint</t>
-        </is>
-      </c>
-      <c r="D47" s="7" t="inlineStr">
-        <is>
-          <t>PK</t>
-        </is>
-      </c>
+          <t>varchar</t>
+        </is>
+      </c>
+      <c r="D47" s="7" t="inlineStr"/>
       <c r="E47" s="7" t="inlineStr">
         <is>
           <t>no</t>
         </is>
       </c>
-      <c r="F47" s="4" t="inlineStr"/>
+      <c r="F47" s="4" t="inlineStr">
+        <is>
+          <t>Hash of the 6-digit code; plain code never stored</t>
+        </is>
+      </c>
     </row>
     <row r="48">
       <c r="A48" s="6" t="inlineStr">
@@ -2244,19 +2235,15 @@
       </c>
       <c r="B48" s="6" t="inlineStr">
         <is>
-          <t>event_registration_id</t>
+          <t>expires_at</t>
         </is>
       </c>
       <c r="C48" s="6" t="inlineStr">
         <is>
-          <t>bigint</t>
-        </is>
-      </c>
-      <c r="D48" s="7" t="inlineStr">
-        <is>
-          <t>FK</t>
-        </is>
-      </c>
+          <t>timestamptz</t>
+        </is>
+      </c>
+      <c r="D48" s="7" t="inlineStr"/>
       <c r="E48" s="7" t="inlineStr">
         <is>
           <t>no</t>
@@ -2264,7 +2251,7 @@
       </c>
       <c r="F48" s="4" t="inlineStr">
         <is>
-          <t>-&gt; event_registrations.id ON DELETE CASCADE</t>
+          <t>TTL from events.otp_ttl_seconds</t>
         </is>
       </c>
     </row>
@@ -2276,12 +2263,12 @@
       </c>
       <c r="B49" s="6" t="inlineStr">
         <is>
-          <t>code_hash</t>
+          <t>attempts</t>
         </is>
       </c>
       <c r="C49" s="6" t="inlineStr">
         <is>
-          <t>varchar</t>
+          <t>smallint</t>
         </is>
       </c>
       <c r="D49" s="7" t="inlineStr"/>
@@ -2292,7 +2279,7 @@
       </c>
       <c r="F49" s="4" t="inlineStr">
         <is>
-          <t>Hash of the 6-digit code; plain code never stored</t>
+          <t>Failed verifications; invalidated at events.otp_max_attempts</t>
         </is>
       </c>
     </row>
@@ -2304,7 +2291,7 @@
       </c>
       <c r="B50" s="6" t="inlineStr">
         <is>
-          <t>expires_at</t>
+          <t>consumed_at</t>
         </is>
       </c>
       <c r="C50" s="6" t="inlineStr">
@@ -2315,12 +2302,12 @@
       <c r="D50" s="7" t="inlineStr"/>
       <c r="E50" s="7" t="inlineStr">
         <is>
-          <t>no</t>
+          <t>yes</t>
         </is>
       </c>
       <c r="F50" s="4" t="inlineStr">
         <is>
-          <t>TTL from events.otp_ttl_seconds</t>
+          <t>Single use</t>
         </is>
       </c>
     </row>
@@ -2332,23 +2319,23 @@
       </c>
       <c r="B51" s="6" t="inlineStr">
         <is>
-          <t>attempts</t>
+          <t>ip</t>
         </is>
       </c>
       <c r="C51" s="6" t="inlineStr">
         <is>
-          <t>smallint</t>
+          <t>inet</t>
         </is>
       </c>
       <c r="D51" s="7" t="inlineStr"/>
       <c r="E51" s="7" t="inlineStr">
         <is>
-          <t>no</t>
+          <t>yes</t>
         </is>
       </c>
       <c r="F51" s="4" t="inlineStr">
         <is>
-          <t>Failed verifications; invalidated at events.otp_max_attempts</t>
+          <t>Requesting IP (rate limit / audit)</t>
         </is>
       </c>
     </row>
@@ -2360,7 +2347,7 @@
       </c>
       <c r="B52" s="6" t="inlineStr">
         <is>
-          <t>consumed_at</t>
+          <t>created_at</t>
         </is>
       </c>
       <c r="C52" s="6" t="inlineStr">
@@ -2371,66 +2358,70 @@
       <c r="D52" s="7" t="inlineStr"/>
       <c r="E52" s="7" t="inlineStr">
         <is>
-          <t>yes</t>
-        </is>
-      </c>
-      <c r="F52" s="4" t="inlineStr">
-        <is>
-          <t>Single use</t>
-        </is>
-      </c>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="F52" s="4" t="inlineStr"/>
     </row>
     <row r="53">
       <c r="A53" s="6" t="inlineStr">
         <is>
-          <t>otp_codes</t>
+          <t>votes</t>
         </is>
       </c>
       <c r="B53" s="6" t="inlineStr">
         <is>
-          <t>ip</t>
+          <t>id</t>
         </is>
       </c>
       <c r="C53" s="6" t="inlineStr">
         <is>
-          <t>inet</t>
-        </is>
-      </c>
-      <c r="D53" s="7" t="inlineStr"/>
+          <t>bigint</t>
+        </is>
+      </c>
+      <c r="D53" s="7" t="inlineStr">
+        <is>
+          <t>PK</t>
+        </is>
+      </c>
       <c r="E53" s="7" t="inlineStr">
         <is>
-          <t>yes</t>
-        </is>
-      </c>
-      <c r="F53" s="4" t="inlineStr">
-        <is>
-          <t>Requesting IP (rate limit / audit)</t>
-        </is>
-      </c>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="F53" s="4" t="inlineStr"/>
     </row>
     <row r="54">
       <c r="A54" s="6" t="inlineStr">
         <is>
-          <t>otp_codes</t>
+          <t>votes</t>
         </is>
       </c>
       <c r="B54" s="6" t="inlineStr">
         <is>
-          <t>created_at</t>
+          <t>event_id</t>
         </is>
       </c>
       <c r="C54" s="6" t="inlineStr">
         <is>
-          <t>timestamptz</t>
-        </is>
-      </c>
-      <c r="D54" s="7" t="inlineStr"/>
+          <t>bigint</t>
+        </is>
+      </c>
+      <c r="D54" s="7" t="inlineStr">
+        <is>
+          <t>FK</t>
+        </is>
+      </c>
       <c r="E54" s="7" t="inlineStr">
         <is>
           <t>no</t>
         </is>
       </c>
-      <c r="F54" s="4" t="inlineStr"/>
+      <c r="F54" s="4" t="inlineStr">
+        <is>
+          <t>Part of both composite FKs</t>
+        </is>
+      </c>
     </row>
     <row r="55">
       <c r="A55" s="6" t="inlineStr">
@@ -2440,7 +2431,7 @@
       </c>
       <c r="B55" s="6" t="inlineStr">
         <is>
-          <t>id</t>
+          <t>visitor_id</t>
         </is>
       </c>
       <c r="C55" s="6" t="inlineStr">
@@ -2450,7 +2441,7 @@
       </c>
       <c r="D55" s="7" t="inlineStr">
         <is>
-          <t>PK</t>
+          <t>FK</t>
         </is>
       </c>
       <c r="E55" s="7" t="inlineStr">
@@ -2458,7 +2449,11 @@
           <t>no</t>
         </is>
       </c>
-      <c r="F55" s="4" t="inlineStr"/>
+      <c r="F55" s="4" t="inlineStr">
+        <is>
+          <t>(event_id, visitor_id) -&gt; event_registrations</t>
+        </is>
+      </c>
     </row>
     <row r="56">
       <c r="A56" s="6" t="inlineStr">
@@ -2468,7 +2463,7 @@
       </c>
       <c r="B56" s="6" t="inlineStr">
         <is>
-          <t>event_id</t>
+          <t>category_id</t>
         </is>
       </c>
       <c r="C56" s="6" t="inlineStr">
@@ -2488,7 +2483,7 @@
       </c>
       <c r="F56" s="4" t="inlineStr">
         <is>
-          <t>Part of both composite FKs</t>
+          <t>(event_id, category_id, exhibitor_id) -&gt; exhibitors(event_id, category_id, id)</t>
         </is>
       </c>
     </row>
@@ -2500,7 +2495,7 @@
       </c>
       <c r="B57" s="6" t="inlineStr">
         <is>
-          <t>visitor_id</t>
+          <t>exhibitor_id</t>
         </is>
       </c>
       <c r="C57" s="6" t="inlineStr">
@@ -2518,11 +2513,7 @@
           <t>no</t>
         </is>
       </c>
-      <c r="F57" s="4" t="inlineStr">
-        <is>
-          <t>(event_id, visitor_id) -&gt; event_registrations</t>
-        </is>
-      </c>
+      <c r="F57" s="4" t="inlineStr"/>
     </row>
     <row r="58">
       <c r="A58" s="6" t="inlineStr">
@@ -2532,27 +2523,23 @@
       </c>
       <c r="B58" s="6" t="inlineStr">
         <is>
-          <t>category_id</t>
+          <t>ip</t>
         </is>
       </c>
       <c r="C58" s="6" t="inlineStr">
         <is>
-          <t>bigint</t>
-        </is>
-      </c>
-      <c r="D58" s="7" t="inlineStr">
-        <is>
-          <t>FK</t>
-        </is>
-      </c>
+          <t>inet</t>
+        </is>
+      </c>
+      <c r="D58" s="7" t="inlineStr"/>
       <c r="E58" s="7" t="inlineStr">
         <is>
-          <t>no</t>
+          <t>yes</t>
         </is>
       </c>
       <c r="F58" s="4" t="inlineStr">
         <is>
-          <t>(event_id, category_id, exhibitor_id) -&gt; category_exhibitor</t>
+          <t>Audit</t>
         </is>
       </c>
     </row>
@@ -2564,19 +2551,15 @@
       </c>
       <c r="B59" s="6" t="inlineStr">
         <is>
-          <t>exhibitor_id</t>
+          <t>created_at</t>
         </is>
       </c>
       <c r="C59" s="6" t="inlineStr">
         <is>
-          <t>bigint</t>
-        </is>
-      </c>
-      <c r="D59" s="7" t="inlineStr">
-        <is>
-          <t>FK</t>
-        </is>
-      </c>
+          <t>timestamptz</t>
+        </is>
+      </c>
+      <c r="D59" s="7" t="inlineStr"/>
       <c r="E59" s="7" t="inlineStr">
         <is>
           <t>no</t>
@@ -2587,48 +2570,52 @@
     <row r="60">
       <c r="A60" s="6" t="inlineStr">
         <is>
-          <t>votes</t>
+          <t>users</t>
         </is>
       </c>
       <c r="B60" s="6" t="inlineStr">
         <is>
-          <t>ip</t>
+          <t>id</t>
         </is>
       </c>
       <c r="C60" s="6" t="inlineStr">
         <is>
-          <t>inet</t>
-        </is>
-      </c>
-      <c r="D60" s="7" t="inlineStr"/>
+          <t>bigint</t>
+        </is>
+      </c>
+      <c r="D60" s="7" t="inlineStr">
+        <is>
+          <t>PK</t>
+        </is>
+      </c>
       <c r="E60" s="7" t="inlineStr">
         <is>
-          <t>yes</t>
-        </is>
-      </c>
-      <c r="F60" s="4" t="inlineStr">
-        <is>
-          <t>Audit</t>
-        </is>
-      </c>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="F60" s="4" t="inlineStr"/>
     </row>
     <row r="61">
       <c r="A61" s="6" t="inlineStr">
         <is>
-          <t>votes</t>
+          <t>users</t>
         </is>
       </c>
       <c r="B61" s="6" t="inlineStr">
         <is>
-          <t>created_at</t>
+          <t>username</t>
         </is>
       </c>
       <c r="C61" s="6" t="inlineStr">
         <is>
-          <t>timestamptz</t>
-        </is>
-      </c>
-      <c r="D61" s="7" t="inlineStr"/>
+          <t>varchar</t>
+        </is>
+      </c>
+      <c r="D61" s="7" t="inlineStr">
+        <is>
+          <t>UNIQUE</t>
+        </is>
+      </c>
       <c r="E61" s="7" t="inlineStr">
         <is>
           <t>no</t>
@@ -2644,25 +2631,25 @@
       </c>
       <c r="B62" s="6" t="inlineStr">
         <is>
-          <t>id</t>
+          <t>password</t>
         </is>
       </c>
       <c r="C62" s="6" t="inlineStr">
         <is>
-          <t>bigint</t>
-        </is>
-      </c>
-      <c r="D62" s="7" t="inlineStr">
-        <is>
-          <t>PK</t>
-        </is>
-      </c>
+          <t>varchar</t>
+        </is>
+      </c>
+      <c r="D62" s="7" t="inlineStr"/>
       <c r="E62" s="7" t="inlineStr">
         <is>
           <t>no</t>
         </is>
       </c>
-      <c r="F62" s="4" t="inlineStr"/>
+      <c r="F62" s="4" t="inlineStr">
+        <is>
+          <t>Bcrypt/Argon2 hash. Admins log in with username + password + TOTP; no email stored</t>
+        </is>
+      </c>
     </row>
     <row r="63">
       <c r="A63" s="6" t="inlineStr">
@@ -2672,25 +2659,25 @@
       </c>
       <c r="B63" s="6" t="inlineStr">
         <is>
-          <t>username</t>
+          <t>app_authentication_secret</t>
         </is>
       </c>
       <c r="C63" s="6" t="inlineStr">
         <is>
-          <t>varchar</t>
-        </is>
-      </c>
-      <c r="D63" s="7" t="inlineStr">
-        <is>
-          <t>UNIQUE</t>
-        </is>
-      </c>
+          <t>text</t>
+        </is>
+      </c>
+      <c r="D63" s="7" t="inlineStr"/>
       <c r="E63" s="7" t="inlineStr">
         <is>
-          <t>no</t>
-        </is>
-      </c>
-      <c r="F63" s="4" t="inlineStr"/>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="F63" s="4" t="inlineStr">
+        <is>
+          <t>TOTP secret for the authenticator app, encrypted (Filament MFA)</t>
+        </is>
+      </c>
     </row>
     <row r="64">
       <c r="A64" s="6" t="inlineStr">
@@ -2700,71 +2687,75 @@
       </c>
       <c r="B64" s="6" t="inlineStr">
         <is>
-          <t>password</t>
+          <t>app_authentication_recovery_codes</t>
         </is>
       </c>
       <c r="C64" s="6" t="inlineStr">
         <is>
-          <t>varchar</t>
+          <t>text</t>
         </is>
       </c>
       <c r="D64" s="7" t="inlineStr"/>
       <c r="E64" s="7" t="inlineStr">
         <is>
-          <t>no</t>
+          <t>yes</t>
         </is>
       </c>
       <c r="F64" s="4" t="inlineStr">
         <is>
-          <t>Bcrypt/Argon2 hash. Admins log in with username + password + TOTP; no email stored</t>
+          <t>One-time recovery codes, encrypted</t>
         </is>
       </c>
     </row>
     <row r="65">
       <c r="A65" s="6" t="inlineStr">
         <is>
-          <t>users</t>
+          <t>audit_logs</t>
         </is>
       </c>
       <c r="B65" s="6" t="inlineStr">
         <is>
-          <t>app_authentication_secret</t>
+          <t>id</t>
         </is>
       </c>
       <c r="C65" s="6" t="inlineStr">
         <is>
-          <t>text</t>
-        </is>
-      </c>
-      <c r="D65" s="7" t="inlineStr"/>
+          <t>bigint</t>
+        </is>
+      </c>
+      <c r="D65" s="7" t="inlineStr">
+        <is>
+          <t>PK</t>
+        </is>
+      </c>
       <c r="E65" s="7" t="inlineStr">
         <is>
-          <t>yes</t>
-        </is>
-      </c>
-      <c r="F65" s="4" t="inlineStr">
-        <is>
-          <t>TOTP secret for the authenticator app, encrypted (Filament MFA)</t>
-        </is>
-      </c>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="F65" s="4" t="inlineStr"/>
     </row>
     <row r="66">
       <c r="A66" s="6" t="inlineStr">
         <is>
-          <t>users</t>
+          <t>audit_logs</t>
         </is>
       </c>
       <c r="B66" s="6" t="inlineStr">
         <is>
-          <t>app_authentication_recovery_codes</t>
+          <t>user_id</t>
         </is>
       </c>
       <c r="C66" s="6" t="inlineStr">
         <is>
-          <t>text</t>
-        </is>
-      </c>
-      <c r="D66" s="7" t="inlineStr"/>
+          <t>bigint</t>
+        </is>
+      </c>
+      <c r="D66" s="7" t="inlineStr">
+        <is>
+          <t>FK</t>
+        </is>
+      </c>
       <c r="E66" s="7" t="inlineStr">
         <is>
           <t>yes</t>
@@ -2772,7 +2763,7 @@
       </c>
       <c r="F66" s="4" t="inlineStr">
         <is>
-          <t>One-time recovery codes, encrypted</t>
+          <t>-&gt; users.id</t>
         </is>
       </c>
     </row>
@@ -2784,7 +2775,7 @@
       </c>
       <c r="B67" s="6" t="inlineStr">
         <is>
-          <t>id</t>
+          <t>event_id</t>
         </is>
       </c>
       <c r="C67" s="6" t="inlineStr">
@@ -2794,15 +2785,19 @@
       </c>
       <c r="D67" s="7" t="inlineStr">
         <is>
-          <t>PK</t>
+          <t>FK</t>
         </is>
       </c>
       <c r="E67" s="7" t="inlineStr">
         <is>
-          <t>no</t>
-        </is>
-      </c>
-      <c r="F67" s="4" t="inlineStr"/>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="F67" s="4" t="inlineStr">
+        <is>
+          <t>-&gt; events.id; null for global actions (e.g. login)</t>
+        </is>
+      </c>
     </row>
     <row r="68">
       <c r="A68" s="6" t="inlineStr">
@@ -2812,27 +2807,23 @@
       </c>
       <c r="B68" s="6" t="inlineStr">
         <is>
-          <t>user_id</t>
+          <t>action</t>
         </is>
       </c>
       <c r="C68" s="6" t="inlineStr">
         <is>
-          <t>bigint</t>
-        </is>
-      </c>
-      <c r="D68" s="7" t="inlineStr">
-        <is>
-          <t>FK</t>
-        </is>
-      </c>
+          <t>varchar</t>
+        </is>
+      </c>
+      <c r="D68" s="7" t="inlineStr"/>
       <c r="E68" s="7" t="inlineStr">
         <is>
-          <t>yes</t>
+          <t>no</t>
         </is>
       </c>
       <c r="F68" s="4" t="inlineStr">
         <is>
-          <t>-&gt; users.id</t>
+          <t>e.g. votes.reset, visitors.export</t>
         </is>
       </c>
     </row>
@@ -2844,19 +2835,15 @@
       </c>
       <c r="B69" s="6" t="inlineStr">
         <is>
-          <t>event_id</t>
+          <t>meta</t>
         </is>
       </c>
       <c r="C69" s="6" t="inlineStr">
         <is>
-          <t>bigint</t>
-        </is>
-      </c>
-      <c r="D69" s="7" t="inlineStr">
-        <is>
-          <t>FK</t>
-        </is>
-      </c>
+          <t>jsonb</t>
+        </is>
+      </c>
+      <c r="D69" s="7" t="inlineStr"/>
       <c r="E69" s="7" t="inlineStr">
         <is>
           <t>yes</t>
@@ -2864,7 +2851,7 @@
       </c>
       <c r="F69" s="4" t="inlineStr">
         <is>
-          <t>-&gt; events.id; null for global actions (e.g. login)</t>
+          <t>Details (old/new values, counts)</t>
         </is>
       </c>
     </row>
@@ -2876,25 +2863,21 @@
       </c>
       <c r="B70" s="6" t="inlineStr">
         <is>
-          <t>action</t>
+          <t>ip</t>
         </is>
       </c>
       <c r="C70" s="6" t="inlineStr">
         <is>
-          <t>varchar</t>
+          <t>inet</t>
         </is>
       </c>
       <c r="D70" s="7" t="inlineStr"/>
       <c r="E70" s="7" t="inlineStr">
         <is>
-          <t>no</t>
-        </is>
-      </c>
-      <c r="F70" s="4" t="inlineStr">
-        <is>
-          <t>e.g. votes.reset, visitors.export</t>
-        </is>
-      </c>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="F70" s="4" t="inlineStr"/>
     </row>
     <row r="71">
       <c r="A71" s="6" t="inlineStr">
@@ -2904,76 +2887,24 @@
       </c>
       <c r="B71" s="6" t="inlineStr">
         <is>
-          <t>meta</t>
+          <t>created_at</t>
         </is>
       </c>
       <c r="C71" s="6" t="inlineStr">
         <is>
-          <t>jsonb</t>
+          <t>timestamptz</t>
         </is>
       </c>
       <c r="D71" s="7" t="inlineStr"/>
       <c r="E71" s="7" t="inlineStr">
         <is>
-          <t>yes</t>
-        </is>
-      </c>
-      <c r="F71" s="4" t="inlineStr">
-        <is>
-          <t>Details (old/new values, counts)</t>
-        </is>
-      </c>
-    </row>
-    <row r="72">
-      <c r="A72" s="6" t="inlineStr">
-        <is>
-          <t>audit_logs</t>
-        </is>
-      </c>
-      <c r="B72" s="6" t="inlineStr">
-        <is>
-          <t>ip</t>
-        </is>
-      </c>
-      <c r="C72" s="6" t="inlineStr">
-        <is>
-          <t>inet</t>
-        </is>
-      </c>
-      <c r="D72" s="7" t="inlineStr"/>
-      <c r="E72" s="7" t="inlineStr">
-        <is>
-          <t>yes</t>
-        </is>
-      </c>
-      <c r="F72" s="4" t="inlineStr"/>
-    </row>
-    <row r="73">
-      <c r="A73" s="6" t="inlineStr">
-        <is>
-          <t>audit_logs</t>
-        </is>
-      </c>
-      <c r="B73" s="6" t="inlineStr">
-        <is>
-          <t>created_at</t>
-        </is>
-      </c>
-      <c r="C73" s="6" t="inlineStr">
-        <is>
-          <t>timestamptz</t>
-        </is>
-      </c>
-      <c r="D73" s="7" t="inlineStr"/>
-      <c r="E73" s="7" t="inlineStr">
-        <is>
-          <t>no</t>
-        </is>
-      </c>
-      <c r="F73" s="4" t="inlineStr"/>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="F71" s="4" t="inlineStr"/>
     </row>
   </sheetData>
-  <autoFilter ref="A1:F73"/>
+  <autoFilter ref="A1:F71"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -2984,7 +2915,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F14"/>
+  <dimension ref="A1:F13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -3190,12 +3121,12 @@
     <row r="7">
       <c r="A7" s="6" t="inlineStr">
         <is>
-          <t>categories</t>
+          <t>visitors</t>
         </is>
       </c>
       <c r="B7" s="6" t="inlineStr">
         <is>
-          <t>category_exhibitor</t>
+          <t>event_registrations</t>
         </is>
       </c>
       <c r="C7" s="7" t="inlineStr">
@@ -3205,29 +3136,29 @@
       </c>
       <c r="D7" s="6" t="inlineStr">
         <is>
-          <t>(event_id, category_id) -&gt; categories(event_id, id)</t>
+          <t>event_registrations.visitor_id</t>
         </is>
       </c>
       <c r="E7" s="4" t="inlineStr">
         <is>
-          <t>CASCADE</t>
+          <t>RESTRICT</t>
         </is>
       </c>
       <c r="F7" s="4" t="inlineStr">
         <is>
-          <t>Same-event guarantee</t>
+          <t>One visitor, many events</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="6" t="inlineStr">
         <is>
-          <t>exhibitors</t>
+          <t>event_registrations</t>
         </is>
       </c>
       <c r="B8" s="6" t="inlineStr">
         <is>
-          <t>category_exhibitor</t>
+          <t>otp_codes</t>
         </is>
       </c>
       <c r="C8" s="7" t="inlineStr">
@@ -3237,7 +3168,7 @@
       </c>
       <c r="D8" s="6" t="inlineStr">
         <is>
-          <t>(event_id, exhibitor_id) -&gt; exhibitors(event_id, id)</t>
+          <t>otp_codes.event_registration_id</t>
         </is>
       </c>
       <c r="E8" s="4" t="inlineStr">
@@ -3247,19 +3178,19 @@
       </c>
       <c r="F8" s="4" t="inlineStr">
         <is>
-          <t>Same-event guarantee</t>
+          <t>OTPs are per event registration</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="6" t="inlineStr">
         <is>
-          <t>visitors</t>
+          <t>event_registrations</t>
         </is>
       </c>
       <c r="B9" s="6" t="inlineStr">
         <is>
-          <t>event_registrations</t>
+          <t>votes</t>
         </is>
       </c>
       <c r="C9" s="7" t="inlineStr">
@@ -3269,7 +3200,7 @@
       </c>
       <c r="D9" s="6" t="inlineStr">
         <is>
-          <t>event_registrations.visitor_id</t>
+          <t>(event_id, visitor_id) -&gt; event_registrations(event_id, visitor_id)</t>
         </is>
       </c>
       <c r="E9" s="4" t="inlineStr">
@@ -3279,19 +3210,19 @@
       </c>
       <c r="F9" s="4" t="inlineStr">
         <is>
-          <t>One visitor, many events</t>
+          <t>Voter must be registered for that event</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="6" t="inlineStr">
         <is>
-          <t>event_registrations</t>
+          <t>categories</t>
         </is>
       </c>
       <c r="B10" s="6" t="inlineStr">
         <is>
-          <t>otp_codes</t>
+          <t>exhibitors</t>
         </is>
       </c>
       <c r="C10" s="7" t="inlineStr">
@@ -3301,24 +3232,24 @@
       </c>
       <c r="D10" s="6" t="inlineStr">
         <is>
-          <t>otp_codes.event_registration_id</t>
+          <t>(event_id, category_id) -&gt; categories(event_id, id)</t>
         </is>
       </c>
       <c r="E10" s="4" t="inlineStr">
         <is>
-          <t>CASCADE</t>
+          <t>RESTRICT</t>
         </is>
       </c>
       <c r="F10" s="4" t="inlineStr">
         <is>
-          <t>OTPs are per event registration</t>
+          <t>Each exhibitor competes in exactly one category of its own event</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="6" t="inlineStr">
         <is>
-          <t>event_registrations</t>
+          <t>exhibitors</t>
         </is>
       </c>
       <c r="B11" s="6" t="inlineStr">
@@ -3333,24 +3264,24 @@
       </c>
       <c r="D11" s="6" t="inlineStr">
         <is>
-          <t>(event_id, visitor_id) -&gt; event_registrations(event_id, visitor_id)</t>
+          <t>(event_id, category_id, exhibitor_id) -&gt; exhibitors(event_id, category_id, id)</t>
         </is>
       </c>
       <c r="E11" s="4" t="inlineStr">
         <is>
-          <t>RESTRICT</t>
+          <t>RESTRICT (delete + update)</t>
         </is>
       </c>
       <c r="F11" s="4" t="inlineStr">
         <is>
-          <t>Voter must be registered for that event</t>
+          <t>Vote only for an exhibitor of that category; exhibitor with votes cannot change category</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="6" t="inlineStr">
         <is>
-          <t>category_exhibitor</t>
+          <t>visitors</t>
         </is>
       </c>
       <c r="B12" s="6" t="inlineStr">
@@ -3365,7 +3296,7 @@
       </c>
       <c r="D12" s="6" t="inlineStr">
         <is>
-          <t>(event_id, category_id, exhibitor_id) -&gt; category_exhibitor</t>
+          <t>votes.visitor_id</t>
         </is>
       </c>
       <c r="E12" s="4" t="inlineStr">
@@ -3375,29 +3306,29 @@
       </c>
       <c r="F12" s="4" t="inlineStr">
         <is>
-          <t>Vote only for an exhibitor entered in that category of that event</t>
+          <t>Votes linked to the visitor (F14)</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="6" t="inlineStr">
         <is>
-          <t>visitors</t>
+          <t>users</t>
         </is>
       </c>
       <c r="B13" s="6" t="inlineStr">
         <is>
-          <t>votes</t>
+          <t>audit_logs</t>
         </is>
       </c>
       <c r="C13" s="7" t="inlineStr">
         <is>
-          <t>1 : N</t>
+          <t>1 : 0..N</t>
         </is>
       </c>
       <c r="D13" s="6" t="inlineStr">
         <is>
-          <t>votes.visitor_id</t>
+          <t>audit_logs.user_id</t>
         </is>
       </c>
       <c r="E13" s="4" t="inlineStr">
@@ -3407,44 +3338,12 @@
       </c>
       <c r="F13" s="4" t="inlineStr">
         <is>
-          <t>Votes linked to the visitor (F14)</t>
-        </is>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" s="6" t="inlineStr">
-        <is>
-          <t>users</t>
-        </is>
-      </c>
-      <c r="B14" s="6" t="inlineStr">
-        <is>
-          <t>audit_logs</t>
-        </is>
-      </c>
-      <c r="C14" s="7" t="inlineStr">
-        <is>
-          <t>1 : 0..N</t>
-        </is>
-      </c>
-      <c r="D14" s="6" t="inlineStr">
-        <is>
-          <t>audit_logs.user_id</t>
-        </is>
-      </c>
-      <c r="E14" s="4" t="inlineStr">
-        <is>
-          <t>RESTRICT</t>
-        </is>
-      </c>
-      <c r="F14" s="4" t="inlineStr">
-        <is>
           <t>Who performed the action</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:F14"/>
+  <autoFilter ref="A1:F13"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -3455,7 +3354,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D19"/>
+  <dimension ref="A1:D18"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="24" customWidth="1" min="1" max="1"/>
@@ -3599,29 +3498,29 @@
     <row r="7">
       <c r="A7" s="6" t="inlineStr">
         <is>
-          <t>category_exhibitor</t>
+          <t>visitors</t>
         </is>
       </c>
       <c r="B7" s="7" t="inlineStr">
         <is>
-          <t>PRIMARY KEY</t>
+          <t>UNIQUE</t>
         </is>
       </c>
       <c r="C7" s="6" t="inlineStr">
         <is>
-          <t>(category_id, exhibitor_id)</t>
+          <t>(phone_hash)</t>
         </is>
       </c>
       <c r="D7" s="4" t="inlineStr">
         <is>
-          <t>An exhibitor is entered in a category once</t>
+          <t>One visitor per phone number (blind index)</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="6" t="inlineStr">
         <is>
-          <t>category_exhibitor</t>
+          <t>event_registrations</t>
         </is>
       </c>
       <c r="B8" s="7" t="inlineStr">
@@ -3631,85 +3530,85 @@
       </c>
       <c r="C8" s="6" t="inlineStr">
         <is>
-          <t>(event_id, category_id, exhibitor_id)</t>
+          <t>(event_id, visitor_id)</t>
         </is>
       </c>
       <c r="D8" s="4" t="inlineStr">
         <is>
-          <t>Target of the votes composite FK</t>
+          <t>One registration per visitor per event; target of the votes FK</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="6" t="inlineStr">
         <is>
-          <t>category_exhibitor</t>
+          <t>otp_codes</t>
         </is>
       </c>
       <c r="B9" s="7" t="inlineStr">
         <is>
-          <t>FOREIGN KEY</t>
+          <t>INDEX</t>
         </is>
       </c>
       <c r="C9" s="6" t="inlineStr">
         <is>
-          <t>(event_id, category_id) -&gt; categories(event_id, id)</t>
+          <t>(event_registration_id, created_at DESC)</t>
         </is>
       </c>
       <c r="D9" s="4" t="inlineStr">
         <is>
-          <t>Category and exhibitor must be in the same event</t>
+          <t>Find the latest active code</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="6" t="inlineStr">
         <is>
-          <t>category_exhibitor</t>
+          <t>votes</t>
         </is>
       </c>
       <c r="B10" s="7" t="inlineStr">
         <is>
-          <t>FOREIGN KEY</t>
+          <t>UNIQUE</t>
         </is>
       </c>
       <c r="C10" s="6" t="inlineStr">
         <is>
-          <t>(event_id, exhibitor_id) -&gt; exhibitors(event_id, id)</t>
+          <t>(visitor_id, category_id)</t>
         </is>
       </c>
       <c r="D10" s="4" t="inlineStr">
         <is>
-          <t>Category and exhibitor must be in the same event</t>
+          <t>ONE VOTE PER CATEGORY per verified phone (F2, F12) - holds under concurrency, retries and multiple instances</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="6" t="inlineStr">
         <is>
-          <t>visitors</t>
+          <t>exhibitors</t>
         </is>
       </c>
       <c r="B11" s="7" t="inlineStr">
         <is>
-          <t>UNIQUE</t>
+          <t>FOREIGN KEY</t>
         </is>
       </c>
       <c r="C11" s="6" t="inlineStr">
         <is>
-          <t>(phone_hash)</t>
+          <t>(event_id, category_id) -&gt; categories(event_id, id)</t>
         </is>
       </c>
       <c r="D11" s="4" t="inlineStr">
         <is>
-          <t>One visitor per phone number (blind index)</t>
+          <t>Category must belong to the exhibitor's own event</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="6" t="inlineStr">
         <is>
-          <t>event_registrations</t>
+          <t>exhibitors</t>
         </is>
       </c>
       <c r="B12" s="7" t="inlineStr">
@@ -3719,56 +3618,56 @@
       </c>
       <c r="C12" s="6" t="inlineStr">
         <is>
-          <t>(event_id, visitor_id)</t>
+          <t>(event_id, category_id, id)</t>
         </is>
       </c>
       <c r="D12" s="4" t="inlineStr">
         <is>
-          <t>One registration per visitor per event; target of the votes FK</t>
+          <t>Target of the votes composite FK</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="6" t="inlineStr">
         <is>
-          <t>otp_codes</t>
+          <t>votes</t>
         </is>
       </c>
       <c r="B13" s="7" t="inlineStr">
         <is>
-          <t>INDEX</t>
+          <t>FOREIGN KEY</t>
         </is>
       </c>
       <c r="C13" s="6" t="inlineStr">
         <is>
-          <t>(event_registration_id, created_at DESC)</t>
+          <t>(event_id, category_id, exhibitor_id) -&gt; exhibitors(event_id, category_id, id) ON UPDATE RESTRICT</t>
         </is>
       </c>
       <c r="D13" s="4" t="inlineStr">
         <is>
-          <t>Find the latest active code</t>
+          <t>Vote must match the exhibitor's category; blocks moving an exhibitor that has votes</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="6" t="inlineStr">
         <is>
-          <t>votes</t>
+          <t>categories</t>
         </is>
       </c>
       <c r="B14" s="7" t="inlineStr">
         <is>
-          <t>UNIQUE</t>
+          <t>MODEL RULE</t>
         </is>
       </c>
       <c r="C14" s="6" t="inlineStr">
         <is>
-          <t>(visitor_id, category_id)</t>
+          <t>max 3 per event (voting.max_categories_per_event)</t>
         </is>
       </c>
       <c r="D14" s="4" t="inlineStr">
         <is>
-          <t>ONE VOTE PER CATEGORY per verified phone (F2, F12) - holds under concurrency, retries and multiple instances</t>
+          <t>Spec: 3 award categories</t>
         </is>
       </c>
     </row>
@@ -3785,12 +3684,12 @@
       </c>
       <c r="C15" s="6" t="inlineStr">
         <is>
-          <t>(event_id, category_id, exhibitor_id) -&gt; category_exhibitor</t>
+          <t>(event_id, visitor_id) -&gt; event_registrations</t>
         </is>
       </c>
       <c r="D15" s="4" t="inlineStr">
         <is>
-          <t>Exhibitor must be entered in that category of that event; blocks un-assigning after votes</t>
+          <t>Voter must be registered for that event (verified state checked in the vote transaction)</t>
         </is>
       </c>
     </row>
@@ -3802,84 +3701,62 @@
       </c>
       <c r="B16" s="7" t="inlineStr">
         <is>
-          <t>FOREIGN KEY</t>
+          <t>INDEX</t>
         </is>
       </c>
       <c r="C16" s="6" t="inlineStr">
         <is>
-          <t>(event_id, visitor_id) -&gt; event_registrations</t>
+          <t>(event_id, category_id, exhibitor_id)</t>
         </is>
       </c>
       <c r="D16" s="4" t="inlineStr">
         <is>
-          <t>Voter must be registered for that event (verified state checked in the vote transaction)</t>
+          <t>Cheap tally queries (COUNT ... GROUP BY)</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="6" t="inlineStr">
         <is>
-          <t>votes</t>
+          <t>users</t>
         </is>
       </c>
       <c r="B17" s="7" t="inlineStr">
         <is>
-          <t>INDEX</t>
+          <t>UNIQUE</t>
         </is>
       </c>
       <c r="C17" s="6" t="inlineStr">
         <is>
-          <t>(event_id, category_id, exhibitor_id)</t>
-        </is>
-      </c>
-      <c r="D17" s="4" t="inlineStr">
-        <is>
-          <t>Cheap tally queries (COUNT ... GROUP BY)</t>
-        </is>
-      </c>
+          <t>(username)</t>
+        </is>
+      </c>
+      <c r="D17" s="4" t="inlineStr"/>
     </row>
     <row r="18">
       <c r="A18" s="6" t="inlineStr">
         <is>
-          <t>users</t>
+          <t>ALL tables</t>
         </is>
       </c>
       <c r="B18" s="7" t="inlineStr">
         <is>
-          <t>UNIQUE</t>
+          <t>SECURITY</t>
         </is>
       </c>
       <c r="C18" s="6" t="inlineStr">
         <is>
-          <t>(username)</t>
-        </is>
-      </c>
-      <c r="D18" s="4" t="inlineStr"/>
-    </row>
-    <row r="19">
-      <c r="A19" s="6" t="inlineStr">
-        <is>
-          <t>ALL tables</t>
-        </is>
-      </c>
-      <c r="B19" s="7" t="inlineStr">
-        <is>
-          <t>SECURITY</t>
-        </is>
-      </c>
-      <c r="C19" s="6" t="inlineStr">
-        <is>
           <t>Row Level Security ENABLED, no policies</t>
         </is>
       </c>
-      <c r="D19" s="4" t="inlineStr">
+      <c r="D18" s="4" t="inlineStr">
         <is>
           <t>Supabase public (anon) API returns nothing; Laravel uses the privileged DB role</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:D19"/>
+  <autoFilter ref="A1:D18"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>